<commit_message>
Update report title (row 1) and as-of date code and tests
</commit_message>
<xml_diff>
--- a/ge/ge_template_ul.xlsx
+++ b/ge/ge_template_ul.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\akohler\projects\LBS\ge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D12B818-DF03-469A-842C-7DEEBABD1AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E808241-FD11-4140-B580-7B56793CF299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="26">
   <si>
     <t>Unit</t>
   </si>
@@ -112,12 +112,6 @@
   </si>
   <si>
     <t>as of 9/30/22</t>
-  </si>
-  <si>
-    <t>GIFTS</t>
-  </si>
-  <si>
-    <t>ENDOWMENTS</t>
   </si>
   <si>
     <t>AUL/UL</t>
@@ -245,7 +239,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -365,13 +359,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -403,22 +406,25 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="4" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -433,11 +439,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -751,52 +757,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="2"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:64" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="J2" s="5" t="s">
@@ -811,43 +815,43 @@
       <c r="M2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="23" t="s">
-        <v>26</v>
+      <c r="N2" s="24" t="s">
+        <v>24</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="O2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="Q2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="17" t="s">
-        <v>27</v>
+      <c r="R2" s="23" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="20" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="17"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="27"/>
+      <c r="R3" s="23"/>
     </row>
     <row r="4" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
@@ -902,7 +906,7 @@
         <v>16</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:64" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23292,14 +23296,8 @@
       <c r="R1121" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
+  <mergeCells count="16">
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="N2:N3"/>
@@ -23308,6 +23306,13 @@
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J3:M3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23341,53 +23346,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="2"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="4"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
     </row>
     <row r="2" spans="1:65" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="J2" s="5" t="s">
@@ -23402,49 +23405,49 @@
       <c r="M2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="23" t="s">
-        <v>26</v>
+      <c r="N2" s="24" t="s">
+        <v>24</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="25" t="s">
+      <c r="R2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="17" t="s">
-        <v>27</v>
+      <c r="S2" s="23" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="20" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="24"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="25"/>
       <c r="O3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="17"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="27"/>
+      <c r="S3" s="23"/>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -23502,7 +23505,7 @@
         <v>16</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:65" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46652,7 +46655,8 @@
       <c r="S1104" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>

</xml_diff>

<commit_message>
DLSR-669: More refinements to GE reports (#116)
* Handle fiscal year end correctly
* Update report title (row 1) and as-of date code and tests
* Move fund_type to GeAccount model
* Update release notes for version 1.3.2
</commit_message>
<xml_diff>
--- a/ge/ge_template_ul.xlsx
+++ b/ge/ge_template_ul.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\akohler\projects\LBS\ge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D12B818-DF03-469A-842C-7DEEBABD1AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E808241-FD11-4140-B580-7B56793CF299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="26">
   <si>
     <t>Unit</t>
   </si>
@@ -112,12 +112,6 @@
   </si>
   <si>
     <t>as of 9/30/22</t>
-  </si>
-  <si>
-    <t>GIFTS</t>
-  </si>
-  <si>
-    <t>ENDOWMENTS</t>
   </si>
   <si>
     <t>AUL/UL</t>
@@ -245,7 +239,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -365,13 +359,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -403,22 +406,25 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="4" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -433,11 +439,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -751,52 +757,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="2"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:64" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="J2" s="5" t="s">
@@ -811,43 +815,43 @@
       <c r="M2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="23" t="s">
-        <v>26</v>
+      <c r="N2" s="24" t="s">
+        <v>24</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="O2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="Q2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="17" t="s">
-        <v>27</v>
+      <c r="R2" s="23" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:64" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="20" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="17"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="27"/>
+      <c r="R3" s="23"/>
     </row>
     <row r="4" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
@@ -902,7 +906,7 @@
         <v>16</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:64" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23292,14 +23296,8 @@
       <c r="R1121" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
+  <mergeCells count="16">
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="N2:N3"/>
@@ -23308,6 +23306,13 @@
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J3:M3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23341,53 +23346,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="2"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="4"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
     </row>
     <row r="2" spans="1:65" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="J2" s="5" t="s">
@@ -23402,49 +23405,49 @@
       <c r="M2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="23" t="s">
-        <v>26</v>
+      <c r="N2" s="24" t="s">
+        <v>24</v>
       </c>
       <c r="O2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="25" t="s">
+      <c r="R2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="17" t="s">
-        <v>27</v>
+      <c r="S2" s="23" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:65" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="20" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="24"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="25"/>
       <c r="O3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="17"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="27"/>
+      <c r="S3" s="23"/>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -23502,7 +23505,7 @@
         <v>16</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:65" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46652,7 +46655,8 @@
       <c r="S1104" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>

</xml_diff>